<commit_message>
feat: upgrade HTML dashboard with audit checksum and git evidence
</commit_message>
<xml_diff>
--- a/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
+++ b/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-25T00:15:56</t>
+          <t>2026-06-25T15:25:42</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-25T00:15:56</t>
+          <t>2026-06-25T15:25:42</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
docs: add Project Phoenix repository baseline and Plutostraat output evidence
</commit_message>
<xml_diff>
--- a/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
+++ b/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-25T15:25:42</t>
+          <t>2026-06-25T16:05:03</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-25T15:25:42</t>
+          <t>2026-06-25T16:05:03</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: add Project Phoenix start dashboard v1.4
</commit_message>
<xml_diff>
--- a/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
+++ b/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-25T16:05:03</t>
+          <t>2026-06-26T13:51:10</t>
         </is>
       </c>
     </row>
@@ -396,12 +396,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -428,12 +428,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -460,12 +460,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -492,12 +492,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -524,12 +524,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -588,12 +588,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -684,12 +684,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -748,12 +748,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -780,12 +780,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -844,12 +844,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -876,12 +876,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-29</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-12-02</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-25T16:05:03</t>
+          <t>2026-06-26T13:51:10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
feat: rebrand Project Phoenix launcher v1.5
</commit_message>
<xml_diff>
--- a/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
+++ b/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-26T13:51:10</t>
+          <t>2026-06-26T14:06:20</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-26T13:51:10</t>
+          <t>2026-06-26T14:06:20</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>

<commit_message>
fix: rebuild HTML dashboard export engine for Project Phoenix v1.6
</commit_message>
<xml_diff>
--- a/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
+++ b/outputs/projects/plutostraat/09_exports/plutostraat_project_tables.xlsx
@@ -156,7 +156,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-26T14:06:20</t>
+          <t>2026-06-26T15:11:00</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-26T14:06:20</t>
+          <t>2026-06-26T15:11:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>